<commit_message>
additional stocks and etfs to watch
</commit_message>
<xml_diff>
--- a/stockwebscrapper/stock_prices.xlsx
+++ b/stockwebscrapper/stock_prices.xlsx
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,438 +413,438 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C29"/>
+  <dimension ref="A1:B36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="B1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>stock</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>price</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="n">
-        <v>0</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>CHR:TSE</t>
+        </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>CHR:TSE</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>$23.04</t>
+          <t>$28.32</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="n">
-        <v>1</v>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>GWO:TSE</t>
+        </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>GWO:TSE</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>$62.04</t>
+          <t>$93.52</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="n">
-        <v>2</v>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>CGX:TSE</t>
+        </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>CGX:TSE</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>$10.50</t>
+          <t>$12.39</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="n">
-        <v>3</v>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>BB:TSE</t>
+        </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>BB:TSE</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>$4.67</t>
+          <t>$11.16</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="n">
-        <v>4</v>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>WCP:TSE</t>
+        </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>WCP:TSE</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>$13.87</t>
+          <t>$18.86</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="n">
-        <v>5</v>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>TLRY:TSE</t>
+        </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>TLRY:TSE</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>$9.83</t>
+          <t>$5.59</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="n">
-        <v>6</v>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>PXT:TSE</t>
+        </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>PXT:TSE</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>$23.15</t>
+          <t>$28.36</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="n">
-        <v>7</v>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>AC:TSE</t>
+        </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>AC:TSE</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>$17.67</t>
+          <t>$28.26</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="n">
-        <v>8</v>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>XMA:TSE</t>
+        </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>XMA:TSE</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>$48.86</t>
+          <t>$48.67</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="n">
-        <v>9</v>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>BEN:NYSE</t>
+        </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>BEN:NYSE</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>$26.24</t>
+          <t>$33.01</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="n">
-        <v>10</v>
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>ACB:TSE</t>
+        </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>ACB:TSE</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>$4.78</t>
+          <t>$5.40</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1" t="n">
-        <v>11</v>
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>OGI:TSE</t>
+        </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
+          <t>$1.44</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>POU:TSE</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>$32.21</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>ASM:TSE</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>$8.94</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>QCLN:NASDAQ</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>$47.82</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>VCNX:OTCMKTS</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>$1.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>AMAT:NASDAQ</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>$444.57</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
           <t>OGI:TSE</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>$2.01</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="1" t="n">
-        <v>12</v>
-      </c>
-      <c r="B14" t="inlineStr">
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>$1.44</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
         <is>
           <t>POU:TSE</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>$29.34</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="1" t="n">
-        <v>13</v>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>ASM:TSE</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>$10.59</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="1" t="n">
-        <v>14</v>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>QCLN:NASDAQ</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>$45.02</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="1" t="n">
-        <v>15</v>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>VCNX:OTCMKTS</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>$0.80</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="1" t="n">
-        <v>16</v>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>AMAT:NASDAQ</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>$324.74</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="1" t="n">
-        <v>17</v>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>OGI:TSE</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>$2.01</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="1" t="n">
-        <v>18</v>
-      </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>POU:TSE</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>$29.34</t>
+          <t>$32.21</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="1" t="n">
-        <v>19</v>
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>QQC:TSE</t>
+        </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>QQC:TSE</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>$39.84</t>
+          <t>$49.31</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="1" t="n">
-        <v>20</v>
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>XUS:TSE</t>
+        </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>XUS:TSE</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>$56.61</t>
+          <t>$66.17</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="1" t="n">
-        <v>21</v>
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>XIC:TSE</t>
+        </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>XIC:TSE</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>$52.93</t>
+          <t>$57.33</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="1" t="n">
-        <v>22</v>
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>XMC:TSE</t>
+        </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>XMC:TSE</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>$35.51</t>
+          <t>$39.24</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="1" t="n">
-        <v>23</v>
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>XHU:TSE</t>
+        </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>XHU:TSE</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>$37.42</t>
+          <t>$41.04</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="1" t="n">
-        <v>24</v>
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>XDIV:TSE</t>
+        </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>XDIV:TSE</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>$38.23</t>
+          <t>$46.31</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="1" t="n">
-        <v>25</v>
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>XEQT:TSE</t>
+        </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>XEQT:TSE</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>$40.24</t>
+          <t>$45.41</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="1" t="n">
-        <v>26</v>
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>VDY:TSE</t>
+        </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>VDY:TSE</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>$65.94</t>
+          <t>$77.17</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="1" t="n">
-        <v>27</v>
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>TGRO:TSE</t>
+        </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>TGRO:TSE</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>$26.64</t>
+          <t>$29.43</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>XEI:TSE</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>$39.75</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>IONQ:NYSE</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>$39.13</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>AKT:TSE</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>$3.81</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>HURA:TSE</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>$47.50</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>ZEQT:TSE</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>$23.39</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>CHPS:TSE</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>$84.14</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>TEC:TSE</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>$62.46</t>
         </is>
       </c>
     </row>

</xml_diff>